<commit_message>
small reward amounts for the intro trails
</commit_message>
<xml_diff>
--- a/PsychoPy/Introtext.xlsx
+++ b/PsychoPy/Introtext.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucas/Documents/Experiments/Mood4/github_Mood4/PsychoPy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7517028-1AC8-A94C-B5D4-23D2B8EF6715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292D8C56-0C01-7E40-8B92-81408F866532}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2980" yWindow="600" windowWidth="41600" windowHeight="22840" xr2:uid="{402AE53E-8E8E-A647-AB36-D93CAEC0D9A2}"/>
   </bookViews>
@@ -32,14 +32,15 @@
     <t>In the next few steps, we will guide you through the task and how it works, you will then do a minimum of 10 practice trials, and finally, you will start the task.</t>
   </si>
   <si>
-    <t>On each trial, you will have the opportunity to earn money by choosing between two options: a guaranteed reward, or a gamble.
-The gamble's probability of winning is indicated by a percentage. Each gamble has two possible outcomes: you either win the indicated reward, or you lose and earn $0.
-On some trials, you will only be shown a single option, which you must select to proceed.</t>
-  </si>
-  <si>
     <t>You will begin the task with $5. The outcome of the choices you make from then on will count for ADDITIONAL money.
 Please select your option by pressing the LEFT or RIGHT arrow key. Once you’ve made your choice, the outcome will be applied to your total.
 On the next screen, you will do a few introductory trials.</t>
+  </si>
+  <si>
+    <t>On each trial, you will have the opportunity to earn money by choosing between two options: a guaranteed reward, or a gamble.
+The gamble's probability of winning is indicated by a percentage. Each gamble has two possible outcomes: you either win the indicated reward, or you lose and earn $0.
+On some trials, you will only be shown a single option, which you must select to proceed.
+While the reward amounts are small, you will complete about 200 trials, and these amounts will quickly add up.</t>
   </si>
 </sst>
 </file>
@@ -936,12 +937,12 @@
     </row>
     <row r="4" spans="1:1" ht="119" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="131" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Moved start_money to 5.5
</commit_message>
<xml_diff>
--- a/PsychoPy/Introtext.xlsx
+++ b/PsychoPy/Introtext.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucas/Documents/Experiments/Mood4/github_Mood4/PsychoPy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{241B897D-5EEF-E04B-A48D-38EAE2F8AA5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8277BD58-EBBF-614D-A8BA-B9EAEEF943AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2980" yWindow="600" windowWidth="41600" windowHeight="22840" xr2:uid="{402AE53E-8E8E-A647-AB36-D93CAEC0D9A2}"/>
   </bookViews>
@@ -32,14 +32,14 @@
     <t>In the next few steps, we will guide you through the task and how it works, you will then do a minimum of 10 practice trials, and finally, you will start the task.</t>
   </si>
   <si>
-    <t>You will begin the task with $5. The outcome of the choices you make from then on will count for ADDITIONAL money.
-Please select your option by pressing the LEFT or RIGHT arrow key. Once you’ve made your choice, the outcome will be applied to your total.
-On the next screen, you will do a few introductory trials.</t>
-  </si>
-  <si>
     <t>On each trial, you will have the opportunity to earn money by choosing between two options: a guaranteed reward, or a gamble.
 The gamble's probability of winning is indicated by a percentage. Each gamble has two possible outcomes: you either win the indicated reward, or you lose and earn $0.
 On some trials, you will only be shown a single option, which you must select to proceed.</t>
+  </si>
+  <si>
+    <t>You will begin the task with $5.50. The outcome of the choices you make from then on will count for ADDITIONAL money.
+Please select your option by pressing the LEFT or RIGHT arrow key. Once you’ve made your choice, the outcome will be applied to your total.
+On the next screen, you will do a few introductory trials.</t>
   </si>
 </sst>
 </file>
@@ -936,12 +936,12 @@
     </row>
     <row r="4" spans="1:1" ht="119" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="131" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>